<commit_message>
Clean up nutrition map data labels and finalize highlight reset logic
</commit_message>
<xml_diff>
--- a/iron-rich-foods_state-wise.xlsx
+++ b/iron-rich-foods_state-wise.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Reps\gene_database_v0_03_dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194D3D2F-FF8F-4044-AE7A-2C0320353645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E533B1C1-1A48-454B-ABE1-DFA13C95DECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1635" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="142">
   <si>
     <t>State</t>
   </si>
@@ -48,9 +48,6 @@
     <t>3.9 mg</t>
   </si>
   <si>
-    <t xml:space="preserve">Ragi sangati </t>
-  </si>
-  <si>
     <t>Fish</t>
   </si>
   <si>
@@ -180,9 +177,6 @@
     <t xml:space="preserve">Seafood based </t>
   </si>
   <si>
-    <t>Ked rice</t>
-  </si>
-  <si>
     <t>1.8 mg</t>
   </si>
   <si>
@@ -354,42 +348,9 @@
     <t>Nagaland</t>
   </si>
   <si>
-    <t xml:space="preserve">Smoked pork </t>
-  </si>
-  <si>
-    <t>Soya beans (fermented)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axone </t>
-  </si>
-  <si>
-    <t>Local greens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boiled vegetables </t>
-  </si>
-  <si>
     <t>Odisha</t>
   </si>
   <si>
-    <t>Finger millet (Mandia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mandia Jau </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saga </t>
-  </si>
-  <si>
-    <t>Small fish</t>
-  </si>
-  <si>
-    <t>1.5 mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Macha Besara </t>
-  </si>
-  <si>
     <t>Punjab</t>
   </si>
   <si>
@@ -432,70 +393,64 @@
     <t>Telangana</t>
   </si>
   <si>
-    <t xml:space="preserve">Pappu koora </t>
-  </si>
-  <si>
-    <t>Mutton/Meat</t>
-  </si>
-  <si>
     <t>Tripura</t>
   </si>
   <si>
-    <t>Bamboo shoots</t>
-  </si>
-  <si>
-    <t>0.5 mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Traditional dishes </t>
-  </si>
-  <si>
     <t>Uttar Pradesh</t>
   </si>
   <si>
     <t>Uttarakhand</t>
   </si>
   <si>
-    <t>Finger millet (Koda)</t>
-  </si>
-  <si>
-    <t>Black soybeans (Bhatt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bhatt ki Churkani </t>
-  </si>
-  <si>
-    <t>Amaranth (Chua)</t>
-  </si>
-  <si>
-    <t>7.5 mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ladoo/Halwa </t>
-  </si>
-  <si>
     <t>West Bengal</t>
   </si>
   <si>
-    <t>1.5-2 mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maurala macher chochori </t>
-  </si>
-  <si>
-    <t>Spinach/Leafy greens</t>
-  </si>
-  <si>
-    <t>2.7-3 mg</t>
-  </si>
-  <si>
-    <t>Lentils (Musur dal)</t>
-  </si>
-  <si>
-    <t>3.1 mg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daily dal </t>
+    <t xml:space="preserve">Ragi Sangati </t>
+  </si>
+  <si>
+    <t>Sesame seeds</t>
+  </si>
+  <si>
+    <t>Pork</t>
+  </si>
+  <si>
+    <t>Smoked</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Mandia Peg</t>
+  </si>
+  <si>
+    <t>Saag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pappu Koora </t>
+  </si>
+  <si>
+    <t>Mandua (Ragi)</t>
+  </si>
+  <si>
+    <t>Jammu and Kashmir</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Kashmiri Rajma</t>
+  </si>
+  <si>
+    <t>Nadru (Lotus Stem)</t>
+  </si>
+  <si>
+    <t>3.6-5 mg</t>
+  </si>
+  <si>
+    <t>1.16-1.17 mg</t>
+  </si>
+  <si>
+    <t>1.51-4.4 mg</t>
   </si>
 </sst>
 </file>
@@ -519,12 +474,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -539,9 +500,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -822,12 +784,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D85"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" customWidth="1"/>
-    <col min="2" max="2" width="20.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.08984375" customWidth="1"/>
+    <col min="1" max="1" width="28.453125" customWidth="1"/>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7265625" customWidth="1"/>
     <col min="4" max="4" width="22.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -856,7 +818,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -864,13 +826,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -878,1147 +840,1189 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D6" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
         <v>23</v>
       </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>24</v>
-      </c>
-      <c r="D8" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
         <v>26</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>27</v>
-      </c>
-      <c r="D9" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
         <v>29</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>30</v>
       </c>
-      <c r="D10" t="s">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="B11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D11" t="s">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" t="s">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
         <v>41</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>42</v>
       </c>
-      <c r="C14" t="s">
-        <v>43</v>
-      </c>
       <c r="D14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" t="s">
         <v>44</v>
-      </c>
-      <c r="D15" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" t="s">
         <v>46</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>47</v>
       </c>
-      <c r="D16" t="s">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="B17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B17" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" t="s">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>49</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="D18" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D18" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" t="s">
-        <v>45</v>
+      <c r="D19" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" t="s">
         <v>55</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
         <v>56</v>
-      </c>
-      <c r="C20" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D21" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B22" t="s">
-        <v>61</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D23" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D22" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>64</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="B24" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C23" t="s">
-        <v>57</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="C24" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>64</v>
-      </c>
-      <c r="B24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24" t="s">
-        <v>68</v>
-      </c>
-    </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="A25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="C25" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" t="s">
         <v>69</v>
       </c>
-      <c r="B26" t="s">
+      <c r="D26" t="s">
         <v>70</v>
-      </c>
-      <c r="C26" t="s">
-        <v>71</v>
-      </c>
-      <c r="D26" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D27" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>135</v>
       </c>
       <c r="B29" t="s">
-        <v>77</v>
+        <v>137</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>139</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>76</v>
+        <v>135</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>138</v>
       </c>
       <c r="C30" t="s">
-        <v>59</v>
+        <v>140</v>
       </c>
       <c r="D30" t="s">
-        <v>37</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>76</v>
+        <v>135</v>
       </c>
       <c r="B31" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" t="s">
+        <v>141</v>
+      </c>
+      <c r="D31" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D34" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="D31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>78</v>
-      </c>
-      <c r="B32" t="s">
-        <v>5</v>
-      </c>
-      <c r="C32" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>78</v>
-      </c>
-      <c r="B33" t="s">
-        <v>80</v>
-      </c>
-      <c r="C33" t="s">
-        <v>81</v>
-      </c>
-      <c r="D33" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>78</v>
-      </c>
-      <c r="B34" t="s">
-        <v>53</v>
-      </c>
-      <c r="C34" t="s">
-        <v>54</v>
-      </c>
-      <c r="D34" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B35" t="s">
-        <v>85</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="D35" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B36" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="C36" t="s">
-        <v>54</v>
+        <v>79</v>
       </c>
       <c r="D36" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
+        <v>76</v>
+      </c>
+      <c r="B37" t="s">
+        <v>51</v>
+      </c>
+      <c r="C37" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B37" t="s">
-        <v>8</v>
-      </c>
-      <c r="C37" t="s">
-        <v>24</v>
-      </c>
-      <c r="D37" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>89</v>
-      </c>
-      <c r="B38" t="s">
-        <v>90</v>
-      </c>
-      <c r="C38" t="s">
-        <v>91</v>
-      </c>
-      <c r="D38" t="s">
-        <v>92</v>
-      </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>89</v>
-      </c>
-      <c r="B39" t="s">
-        <v>46</v>
-      </c>
-      <c r="C39" t="s">
-        <v>47</v>
-      </c>
-      <c r="D39" t="s">
-        <v>48</v>
+      <c r="A39" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>89</v>
-      </c>
-      <c r="B40" t="s">
-        <v>36</v>
-      </c>
-      <c r="C40" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" t="s">
-        <v>45</v>
+      <c r="A40" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B41" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C41" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D41" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B42" t="s">
-        <v>97</v>
+        <v>45</v>
       </c>
       <c r="C42" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="D42" t="s">
-        <v>98</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" t="s">
+        <v>35</v>
+      </c>
+      <c r="C43" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B43" t="s">
-        <v>11</v>
-      </c>
-      <c r="C43" t="s">
-        <v>59</v>
-      </c>
-      <c r="D43" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>99</v>
-      </c>
-      <c r="B44" t="s">
-        <v>100</v>
-      </c>
-      <c r="C44" t="s">
-        <v>75</v>
-      </c>
-      <c r="D44" t="s">
-        <v>101</v>
+      <c r="D44" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>99</v>
-      </c>
-      <c r="B45" t="s">
-        <v>11</v>
-      </c>
-      <c r="C45" t="s">
-        <v>59</v>
-      </c>
-      <c r="D45" t="s">
-        <v>19</v>
+      <c r="A45" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>99</v>
-      </c>
-      <c r="B46" t="s">
-        <v>8</v>
-      </c>
-      <c r="C46" t="s">
-        <v>24</v>
-      </c>
-      <c r="D46" t="s">
-        <v>102</v>
+      <c r="A46" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B47" t="s">
-        <v>29</v>
+        <v>98</v>
       </c>
       <c r="C47" t="s">
-        <v>30</v>
+        <v>73</v>
       </c>
       <c r="D47" t="s">
-        <v>17</v>
+        <v>99</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B48" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C48" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="D48" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
+        <v>97</v>
+      </c>
+      <c r="B49" t="s">
+        <v>7</v>
+      </c>
+      <c r="C49" t="s">
+        <v>23</v>
+      </c>
+      <c r="D49" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="B49" t="s">
-        <v>104</v>
-      </c>
-      <c r="C49" t="s">
-        <v>59</v>
-      </c>
-      <c r="D49" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>106</v>
-      </c>
-      <c r="B50" t="s">
-        <v>11</v>
-      </c>
-      <c r="C50" t="s">
-        <v>59</v>
-      </c>
-      <c r="D50" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>106</v>
-      </c>
-      <c r="B51" t="s">
-        <v>46</v>
-      </c>
-      <c r="C51" t="s">
-        <v>47</v>
-      </c>
-      <c r="D51" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>106</v>
-      </c>
-      <c r="B52" t="s">
-        <v>8</v>
-      </c>
-      <c r="C52" t="s">
-        <v>24</v>
-      </c>
-      <c r="D52" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B53" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="D53" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B54" t="s">
-        <v>110</v>
+        <v>45</v>
       </c>
       <c r="C54" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="D54" t="s">
-        <v>111</v>
+        <v>47</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B55" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="C55" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="D55" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>114</v>
-      </c>
-      <c r="B56" t="s">
-        <v>115</v>
-      </c>
-      <c r="C56" t="s">
-        <v>6</v>
-      </c>
-      <c r="D56" t="s">
-        <v>116</v>
+      <c r="A56" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>114</v>
-      </c>
-      <c r="B57" t="s">
-        <v>53</v>
-      </c>
-      <c r="C57" t="s">
-        <v>54</v>
-      </c>
-      <c r="D57" t="s">
-        <v>117</v>
+      <c r="A57" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>114</v>
-      </c>
-      <c r="B58" t="s">
-        <v>118</v>
-      </c>
-      <c r="C58" t="s">
-        <v>119</v>
-      </c>
-      <c r="D58" t="s">
-        <v>120</v>
+      <c r="A58" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="B59" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="C59" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="D59" t="s">
-        <v>37</v>
+        <v>131</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="B60" t="s">
-        <v>67</v>
+        <v>10</v>
       </c>
       <c r="C60" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D60" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="B61" t="s">
+        <v>7</v>
+      </c>
+      <c r="C61" t="s">
+        <v>23</v>
+      </c>
+      <c r="D61" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D64" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D61" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>123</v>
-      </c>
-      <c r="B62" t="s">
-        <v>65</v>
-      </c>
-      <c r="C62" t="s">
-        <v>57</v>
-      </c>
-      <c r="D62" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>123</v>
-      </c>
-      <c r="B63" t="s">
-        <v>124</v>
-      </c>
-      <c r="C63" t="s">
-        <v>125</v>
-      </c>
-      <c r="D63" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>123</v>
-      </c>
-      <c r="B64" t="s">
-        <v>61</v>
-      </c>
-      <c r="C64" t="s">
-        <v>62</v>
-      </c>
-      <c r="D64" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="B65" t="s">
-        <v>128</v>
+        <v>63</v>
       </c>
       <c r="C65" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D65" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="B66" t="s">
-        <v>11</v>
+        <v>111</v>
       </c>
       <c r="C66" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="D66" t="s">
-        <v>19</v>
+        <v>90</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="B67" t="s">
+        <v>59</v>
+      </c>
+      <c r="C67" t="s">
+        <v>60</v>
+      </c>
+      <c r="D67" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C70" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D70" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="D67" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
-        <v>130</v>
-      </c>
-      <c r="B68" t="s">
-        <v>5</v>
-      </c>
-      <c r="C68" t="s">
-        <v>6</v>
-      </c>
-      <c r="D68" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>130</v>
-      </c>
-      <c r="B69" t="s">
-        <v>53</v>
-      </c>
-      <c r="C69" t="s">
-        <v>54</v>
-      </c>
-      <c r="D69" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>130</v>
-      </c>
-      <c r="B70" t="s">
-        <v>80</v>
-      </c>
-      <c r="C70" t="s">
-        <v>81</v>
-      </c>
-      <c r="D70" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="B71" t="s">
-        <v>94</v>
+        <v>5</v>
       </c>
       <c r="C71" t="s">
-        <v>95</v>
+        <v>6</v>
       </c>
       <c r="D71" t="s">
-        <v>66</v>
+        <v>118</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="B72" t="s">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="C72" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D72" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="B73" t="s">
-        <v>136</v>
+        <v>78</v>
       </c>
       <c r="C73" t="s">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="D73" t="s">
-        <v>88</v>
+        <v>120</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>137</v>
-      </c>
-      <c r="B74" t="s">
-        <v>8</v>
-      </c>
-      <c r="C74" t="s">
-        <v>24</v>
-      </c>
-      <c r="D74" t="s">
-        <v>35</v>
+      <c r="A74" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>137</v>
-      </c>
-      <c r="B75" t="s">
-        <v>11</v>
-      </c>
-      <c r="C75" t="s">
-        <v>59</v>
-      </c>
-      <c r="D75" t="s">
-        <v>19</v>
+      <c r="A75" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>137</v>
-      </c>
-      <c r="B76" t="s">
-        <v>138</v>
-      </c>
-      <c r="C76" t="s">
-        <v>139</v>
-      </c>
-      <c r="D76" t="s">
-        <v>140</v>
+      <c r="A76" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
       <c r="B77" t="s">
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="C77" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="D77" t="s">
-        <v>66</v>
+        <v>132</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
       <c r="B78" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C78" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="D78" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
       <c r="B79" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="C79" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="D79" t="s">
-        <v>40</v>
+        <v>130</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>142</v>
-      </c>
-      <c r="B80" t="s">
-        <v>143</v>
-      </c>
-      <c r="C80" t="s">
-        <v>6</v>
-      </c>
-      <c r="D80" t="s">
+      <c r="A80" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D81" s="2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
-        <v>142</v>
-      </c>
-      <c r="B81" t="s">
-        <v>144</v>
-      </c>
-      <c r="C81" t="s">
-        <v>91</v>
-      </c>
-      <c r="D81" t="s">
-        <v>145</v>
-      </c>
-    </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
-        <v>142</v>
-      </c>
-      <c r="B82" t="s">
-        <v>146</v>
-      </c>
-      <c r="C82" t="s">
-        <v>147</v>
-      </c>
-      <c r="D82" t="s">
-        <v>148</v>
+      <c r="A82" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="B83" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="C83" t="s">
-        <v>150</v>
+        <v>6</v>
       </c>
       <c r="D83" t="s">
-        <v>151</v>
+        <v>64</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="B84" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="C84" t="s">
-        <v>153</v>
+        <v>57</v>
       </c>
       <c r="D84" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="B85" t="s">
-        <v>154</v>
+        <v>45</v>
       </c>
       <c r="C85" t="s">
-        <v>155</v>
+        <v>46</v>
       </c>
       <c r="D85" t="s">
-        <v>156</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Oncology Map with top 10 incidence rates and gradient. Hide numbers for other states.
</commit_message>
<xml_diff>
--- a/iron-rich-foods_state-wise.xlsx
+++ b/iron-rich-foods_state-wise.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Reps\gene_database_v0_03_dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FD762A5-195A-4CDB-9F2C-2446051F87AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E500B2CF-C7CC-4946-9FE5-0C23E866E862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-1635" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Iron Rich Foods" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Iron Rich Foods'!$A$1:$D$217</definedName>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="957" uniqueCount="126">
   <si>
     <t>State / UT</t>
   </si>
@@ -296,13 +297,118 @@
   </si>
   <si>
     <t>Andaman and Nicobar Islands</t>
+  </si>
+  <si>
+    <t>All numbers in Rs Cr unless otherwise specified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P&amp;L Heads </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 0 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 4 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 6 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 7 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 8 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 9 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yr 10 </t>
+  </si>
+  <si>
+    <t>Census Beds (Nos)</t>
+  </si>
+  <si>
+    <t>% Occupied</t>
+  </si>
+  <si>
+    <t>ARPOB</t>
+  </si>
+  <si>
+    <t>NET Revenue</t>
+  </si>
+  <si>
+    <t>Growth</t>
+  </si>
+  <si>
+    <t>GROSS CONTRIBUTION</t>
+  </si>
+  <si>
+    <t>% of Net Revenue</t>
+  </si>
+  <si>
+    <t>EBDITAR</t>
+  </si>
+  <si>
+    <t>BT FEE</t>
+  </si>
+  <si>
+    <t>EBDITA</t>
+  </si>
+  <si>
+    <t>NET PROFIT (PBT)</t>
+  </si>
+  <si>
+    <t>Cash from Operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- </t>
+  </si>
+  <si>
+    <t>Change in NWC</t>
+  </si>
+  <si>
+    <t>Capex - Civil + Others</t>
+  </si>
+  <si>
+    <t>Capex - Med Eqpmt</t>
+  </si>
+  <si>
+    <t>Terminal Value</t>
+  </si>
+  <si>
+    <t>FCF</t>
+  </si>
+  <si>
+    <t>Interest</t>
+  </si>
+  <si>
+    <t>Funding Required for Business</t>
+  </si>
+  <si>
+    <t>ROCE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -315,13 +421,66 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFC00000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -343,8 +502,14 @@
         <fgColor rgb="FFFFF3E0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -367,11 +532,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -398,6 +578,48 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3835,4 +4057,962 @@
   <autoFilter ref="A1:D217" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F1F8C9D-486D-4238-B573-C6066853DFC8}">
+  <dimension ref="A1:M26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.6328125" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="H2" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="J2" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="K2" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="L2" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="M2" s="21" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="13">
+        <v>0</v>
+      </c>
+      <c r="E3" s="13">
+        <v>0</v>
+      </c>
+      <c r="F3" s="13">
+        <v>0</v>
+      </c>
+      <c r="G3" s="13">
+        <v>0</v>
+      </c>
+      <c r="H3" s="13">
+        <v>0</v>
+      </c>
+      <c r="I3" s="13">
+        <v>0</v>
+      </c>
+      <c r="J3" s="13">
+        <v>0</v>
+      </c>
+      <c r="K3" s="13">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13">
+        <v>0</v>
+      </c>
+      <c r="M3" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A4" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="14">
+        <v>0</v>
+      </c>
+      <c r="E4" s="14">
+        <v>0</v>
+      </c>
+      <c r="F4" s="14">
+        <v>0</v>
+      </c>
+      <c r="G4" s="14">
+        <v>0</v>
+      </c>
+      <c r="H4" s="14">
+        <v>0</v>
+      </c>
+      <c r="I4" s="14">
+        <v>0</v>
+      </c>
+      <c r="J4" s="14">
+        <v>0</v>
+      </c>
+      <c r="K4" s="14">
+        <v>0</v>
+      </c>
+      <c r="L4" s="14">
+        <v>0</v>
+      </c>
+      <c r="M4" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="13">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
+        <v>0</v>
+      </c>
+      <c r="I5" s="13">
+        <v>0</v>
+      </c>
+      <c r="J5" s="13">
+        <v>0</v>
+      </c>
+      <c r="K5" s="13">
+        <v>0</v>
+      </c>
+      <c r="L5" s="13">
+        <v>0</v>
+      </c>
+      <c r="M5" s="13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A6" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21">
+        <v>0</v>
+      </c>
+      <c r="D6" s="21">
+        <v>28.5</v>
+      </c>
+      <c r="E6" s="21">
+        <v>31</v>
+      </c>
+      <c r="F6" s="21">
+        <v>37</v>
+      </c>
+      <c r="G6" s="21">
+        <v>45</v>
+      </c>
+      <c r="H6" s="21">
+        <v>54</v>
+      </c>
+      <c r="I6" s="21">
+        <v>66</v>
+      </c>
+      <c r="J6" s="21">
+        <v>81</v>
+      </c>
+      <c r="K6" s="21">
+        <v>99</v>
+      </c>
+      <c r="L6" s="21">
+        <v>121</v>
+      </c>
+      <c r="M6" s="21">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" s="15"/>
+      <c r="B7" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="F7" s="17">
+        <v>0.16900000000000001</v>
+      </c>
+      <c r="G7" s="17">
+        <v>0.218</v>
+      </c>
+      <c r="H7" s="17">
+        <v>0.219</v>
+      </c>
+      <c r="I7" s="17">
+        <v>0.221</v>
+      </c>
+      <c r="J7" s="17">
+        <v>0.221</v>
+      </c>
+      <c r="K7" s="17">
+        <v>0.222</v>
+      </c>
+      <c r="L7" s="17">
+        <v>0.223</v>
+      </c>
+      <c r="M7" s="17">
+        <v>0.224</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21">
+        <v>0</v>
+      </c>
+      <c r="D8" s="21">
+        <v>27</v>
+      </c>
+      <c r="E8" s="21">
+        <v>29</v>
+      </c>
+      <c r="F8" s="21">
+        <v>34</v>
+      </c>
+      <c r="G8" s="21">
+        <v>42</v>
+      </c>
+      <c r="H8" s="21">
+        <v>51</v>
+      </c>
+      <c r="I8" s="21">
+        <v>63</v>
+      </c>
+      <c r="J8" s="21">
+        <v>77</v>
+      </c>
+      <c r="K8" s="21">
+        <v>94</v>
+      </c>
+      <c r="L8" s="21">
+        <v>115</v>
+      </c>
+      <c r="M8" s="21">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="18"/>
+      <c r="B9" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="16"/>
+      <c r="D9" s="17">
+        <v>0.93200000000000005</v>
+      </c>
+      <c r="E9" s="17">
+        <v>0.93200000000000005</v>
+      </c>
+      <c r="F9" s="17">
+        <v>0.93400000000000005</v>
+      </c>
+      <c r="G9" s="17">
+        <v>0.93600000000000005</v>
+      </c>
+      <c r="H9" s="17">
+        <v>0.93899999999999995</v>
+      </c>
+      <c r="I9" s="17">
+        <v>0.94099999999999995</v>
+      </c>
+      <c r="J9" s="17">
+        <v>0.94299999999999995</v>
+      </c>
+      <c r="K9" s="17">
+        <v>0.94399999999999995</v>
+      </c>
+      <c r="L9" s="17">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="M9" s="17">
+        <v>0.94699999999999995</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A10" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21">
+        <v>16.7</v>
+      </c>
+      <c r="E10" s="21">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="F10" s="21">
+        <v>11.9</v>
+      </c>
+      <c r="G10" s="21">
+        <v>18.3</v>
+      </c>
+      <c r="H10" s="21">
+        <v>26.1</v>
+      </c>
+      <c r="I10" s="21">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="J10" s="21">
+        <v>47.7</v>
+      </c>
+      <c r="K10" s="21">
+        <v>62.5</v>
+      </c>
+      <c r="L10" s="21">
+        <v>80.7</v>
+      </c>
+      <c r="M10" s="21">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="18"/>
+      <c r="B11" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="16"/>
+      <c r="D11" s="17">
+        <v>0.58499999999999996</v>
+      </c>
+      <c r="E11" s="17">
+        <v>0.61</v>
+      </c>
+      <c r="F11" s="17">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="G11" s="17">
+        <v>0.40899999999999997</v>
+      </c>
+      <c r="H11" s="17">
+        <v>0.47899999999999998</v>
+      </c>
+      <c r="I11" s="17">
+        <v>0.53800000000000003</v>
+      </c>
+      <c r="J11" s="17">
+        <v>0.58799999999999997</v>
+      </c>
+      <c r="K11" s="17">
+        <v>0.629</v>
+      </c>
+      <c r="L11" s="17">
+        <v>0.66500000000000004</v>
+      </c>
+      <c r="M11" s="17">
+        <v>0.69499999999999995</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A12" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21">
+        <v>0</v>
+      </c>
+      <c r="E12" s="21">
+        <v>0</v>
+      </c>
+      <c r="F12" s="21">
+        <v>0</v>
+      </c>
+      <c r="G12" s="21">
+        <v>0</v>
+      </c>
+      <c r="H12" s="21">
+        <v>0</v>
+      </c>
+      <c r="I12" s="21">
+        <v>0</v>
+      </c>
+      <c r="J12" s="21">
+        <v>0</v>
+      </c>
+      <c r="K12" s="21">
+        <v>0</v>
+      </c>
+      <c r="L12" s="21">
+        <v>0</v>
+      </c>
+      <c r="M12" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="18"/>
+      <c r="B13" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17">
+        <v>0</v>
+      </c>
+      <c r="E13" s="17">
+        <v>0</v>
+      </c>
+      <c r="F13" s="17">
+        <v>0</v>
+      </c>
+      <c r="G13" s="17">
+        <v>0</v>
+      </c>
+      <c r="H13" s="17">
+        <v>0</v>
+      </c>
+      <c r="I13" s="17">
+        <v>0</v>
+      </c>
+      <c r="J13" s="17">
+        <v>0</v>
+      </c>
+      <c r="K13" s="17">
+        <v>0</v>
+      </c>
+      <c r="L13" s="17">
+        <v>0</v>
+      </c>
+      <c r="M13" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21">
+        <v>16.670000000000002</v>
+      </c>
+      <c r="E14" s="21">
+        <v>19.13</v>
+      </c>
+      <c r="F14" s="21">
+        <v>11.93</v>
+      </c>
+      <c r="G14" s="21">
+        <v>18.260000000000002</v>
+      </c>
+      <c r="H14" s="21">
+        <v>26.08</v>
+      </c>
+      <c r="I14" s="21">
+        <v>35.75</v>
+      </c>
+      <c r="J14" s="21">
+        <v>47.71</v>
+      </c>
+      <c r="K14" s="21">
+        <v>62.46</v>
+      </c>
+      <c r="L14" s="21">
+        <v>80.680000000000007</v>
+      </c>
+      <c r="M14" s="21">
+        <v>103.19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="18"/>
+      <c r="B15" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17">
+        <v>0.58499999999999996</v>
+      </c>
+      <c r="E15" s="17">
+        <v>0.61</v>
+      </c>
+      <c r="F15" s="17">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="G15" s="17">
+        <v>0.40899999999999997</v>
+      </c>
+      <c r="H15" s="17">
+        <v>0.47899999999999998</v>
+      </c>
+      <c r="I15" s="17">
+        <v>0.53800000000000003</v>
+      </c>
+      <c r="J15" s="17">
+        <v>0.58799999999999997</v>
+      </c>
+      <c r="K15" s="17">
+        <v>0.629</v>
+      </c>
+      <c r="L15" s="17">
+        <v>0.66500000000000004</v>
+      </c>
+      <c r="M15" s="17">
+        <v>0.69499999999999995</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21">
+        <v>-17.920000000000002</v>
+      </c>
+      <c r="E16" s="21">
+        <v>-11.9</v>
+      </c>
+      <c r="F16" s="21">
+        <v>-15.53</v>
+      </c>
+      <c r="G16" s="21">
+        <v>-5.64</v>
+      </c>
+      <c r="H16" s="21">
+        <v>5.75</v>
+      </c>
+      <c r="I16" s="21">
+        <v>17.97</v>
+      </c>
+      <c r="J16" s="21">
+        <v>29.93</v>
+      </c>
+      <c r="K16" s="21">
+        <v>44.68</v>
+      </c>
+      <c r="L16" s="21">
+        <v>62.9</v>
+      </c>
+      <c r="M16" s="21">
+        <v>85.41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" s="18"/>
+      <c r="B17" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="19"/>
+      <c r="D17" s="17">
+        <v>-0.629</v>
+      </c>
+      <c r="E17" s="17">
+        <v>-0.379</v>
+      </c>
+      <c r="F17" s="17">
+        <v>-0.42399999999999999</v>
+      </c>
+      <c r="G17" s="17">
+        <v>-0.126</v>
+      </c>
+      <c r="H17" s="17">
+        <v>0.106</v>
+      </c>
+      <c r="I17" s="17">
+        <v>0.27</v>
+      </c>
+      <c r="J17" s="17">
+        <v>0.36899999999999999</v>
+      </c>
+      <c r="K17" s="17">
+        <v>0.45</v>
+      </c>
+      <c r="L17" s="17">
+        <v>0.51800000000000002</v>
+      </c>
+      <c r="M17" s="17">
+        <v>0.57499999999999996</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="D18" s="13">
+        <v>16.670000000000002</v>
+      </c>
+      <c r="E18" s="13">
+        <v>19.07</v>
+      </c>
+      <c r="F18" s="13">
+        <v>11.99</v>
+      </c>
+      <c r="G18" s="13">
+        <v>18.260000000000002</v>
+      </c>
+      <c r="H18" s="13">
+        <v>25.28</v>
+      </c>
+      <c r="I18" s="13">
+        <v>31.23</v>
+      </c>
+      <c r="J18" s="13">
+        <v>40.17</v>
+      </c>
+      <c r="K18" s="13">
+        <v>51.21</v>
+      </c>
+      <c r="L18" s="13">
+        <v>64.849999999999994</v>
+      </c>
+      <c r="M18" s="13">
+        <v>81.69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="D19" s="13">
+        <v>-1.92</v>
+      </c>
+      <c r="E19" s="13">
+        <v>-0.19</v>
+      </c>
+      <c r="F19" s="13">
+        <v>-0.37</v>
+      </c>
+      <c r="G19" s="13">
+        <v>-0.56000000000000005</v>
+      </c>
+      <c r="H19" s="13">
+        <v>-0.68</v>
+      </c>
+      <c r="I19" s="13">
+        <v>-0.84</v>
+      </c>
+      <c r="J19" s="13">
+        <v>-1.03</v>
+      </c>
+      <c r="K19" s="13">
+        <v>-1.27</v>
+      </c>
+      <c r="L19" s="13">
+        <v>-1.56</v>
+      </c>
+      <c r="M19" s="13">
+        <v>-1.92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="C20" s="13">
+        <v>-15</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="I20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="K20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="L20" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="M20" s="13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="13">
+        <v>-224.72</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="I21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="J21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="K21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="L21" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="M21" s="13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" s="12"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="20">
+        <v>1185.2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A23" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21">
+        <v>-239.72</v>
+      </c>
+      <c r="D23" s="21">
+        <v>14.76</v>
+      </c>
+      <c r="E23" s="21">
+        <v>18.88</v>
+      </c>
+      <c r="F23" s="21">
+        <v>11.63</v>
+      </c>
+      <c r="G23" s="21">
+        <v>17.7</v>
+      </c>
+      <c r="H23" s="21">
+        <v>24.61</v>
+      </c>
+      <c r="I23" s="21">
+        <v>30.38</v>
+      </c>
+      <c r="J23" s="21">
+        <v>39.14</v>
+      </c>
+      <c r="K23" s="21">
+        <v>49.94</v>
+      </c>
+      <c r="L23" s="21">
+        <v>63.29</v>
+      </c>
+      <c r="M23" s="22">
+        <v>1264.97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A24" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12">
+        <v>-20.38</v>
+      </c>
+      <c r="D24" s="12">
+        <v>-16.809999999999999</v>
+      </c>
+      <c r="E24" s="12">
+        <v>-13.25</v>
+      </c>
+      <c r="F24" s="12">
+        <v>-9.68</v>
+      </c>
+      <c r="G24" s="12">
+        <v>-6.12</v>
+      </c>
+      <c r="H24" s="12">
+        <v>-2.56</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="L24" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="M24" s="12" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21">
+        <v>-260.08999999999997</v>
+      </c>
+      <c r="D25" s="21">
+        <v>-2.06</v>
+      </c>
+      <c r="E25" s="21">
+        <v>5.63</v>
+      </c>
+      <c r="F25" s="21">
+        <v>1.94</v>
+      </c>
+      <c r="G25" s="21">
+        <v>11.58</v>
+      </c>
+      <c r="H25" s="21">
+        <v>22.05</v>
+      </c>
+      <c r="I25" s="21">
+        <v>30.38</v>
+      </c>
+      <c r="J25" s="21">
+        <v>39.14</v>
+      </c>
+      <c r="K25" s="21">
+        <v>49.94</v>
+      </c>
+      <c r="L25" s="21">
+        <v>63.29</v>
+      </c>
+      <c r="M25" s="22">
+        <v>1264.97</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A26" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="23">
+        <v>-5.0000000000000001E-3</v>
+      </c>
+      <c r="E26" s="23">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="F26" s="23">
+        <v>-2.4E-2</v>
+      </c>
+      <c r="G26" s="23">
+        <v>2E-3</v>
+      </c>
+      <c r="H26" s="23">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="I26" s="23">
+        <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="J26" s="23">
+        <v>0.123</v>
+      </c>
+      <c r="K26" s="23">
+        <v>0.182</v>
+      </c>
+      <c r="L26" s="23">
+        <v>0.255</v>
+      </c>
+      <c r="M26" s="23">
+        <v>0.34399999999999997</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>